<commit_message>
Add Salutation as new feature
</commit_message>
<xml_diff>
--- a/storage/app/templates/import_leads_template.xlsx
+++ b/storage/app/templates/import_leads_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
   <si>
     <t>Organization Name</t>
   </si>
@@ -23,6 +23,9 @@
     <t>MD/CEO</t>
   </si>
   <si>
+    <t>Salutation</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -38,6 +41,9 @@
     <t>Mr. Fahim Sinha</t>
   </si>
   <si>
+    <t>Bhai</t>
+  </si>
+  <si>
     <t>sample.ceo@example.com</t>
   </si>
   <si>
@@ -51,6 +57,9 @@
   </si>
   <si>
     <t>Ms. Example Contact</t>
+  </si>
+  <si>
+    <t>Apu</t>
   </si>
   <si>
     <t>contact@example.com</t>
@@ -67,18 +76,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="1"/>
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
@@ -107,9 +107,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,65 +408,67 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col min="1" max="1" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="39.99" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="61.271" bestFit="true" customWidth="true" style="0"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add CC email support to lead import flow
Extends lead import to recognize, validate, and store a new `CC Email` column from CSV/XLSX templates, including missing-data checks and updated UI/template guidance. Outreach address resolution now auto-includes imported non-primary lead emails in CC while preserving deduplication with manually submitted CC recipients.
</commit_message>
<xml_diff>
--- a/storage/app/templates/import_leads_template.xlsx
+++ b/storage/app/templates/import_leads_template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
   <si>
     <t>Organization Name</t>
   </si>
@@ -29,6 +29,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>CC</t>
+  </si>
+  <si>
     <t>Cell/Phone</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
     <t>sample.ceo@example.com</t>
   </si>
   <si>
+    <t>assistant@example.com</t>
+  </si>
+  <si>
     <t>+880 17XX-XXXXXX</t>
   </si>
   <si>
@@ -63,6 +69,9 @@
   </si>
   <si>
     <t>contact@example.com</t>
+  </si>
+  <si>
+    <t>cc1@example.com, cc2@example.com</t>
   </si>
   <si>
     <t>+880 17XX-XXXXXX / +880 2-XXXXXXX</t>
@@ -408,10 +417,19 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="31.707" bestFit="true" customWidth="true" style="0"/>
+    <col min="2" max="2" width="23.423" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="26.993" bestFit="true" customWidth="true" style="0"/>
+    <col min="5" max="5" width="38.848" bestFit="true" customWidth="true" style="0"/>
+    <col min="6" max="6" width="39.99" bestFit="true" customWidth="true" style="0"/>
+    <col min="7" max="7" width="61.271" bestFit="true" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -430,45 +448,54 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>